<commit_message>
added missing MSH3 frameshift
</commit_message>
<xml_diff>
--- a/Sup Tables/table-s9.xlsx
+++ b/Sup Tables/table-s9.xlsx
@@ -51,6 +51,7 @@
         <sz val="11"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">（</t>
     </r>
@@ -82,6 +83,7 @@
         <sz val="11"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">（</t>
     </r>
@@ -301,7 +303,7 @@
     <t xml:space="preserve">p.Ala154Thr</t>
   </si>
   <si>
-    <t xml:space="preserve">p.Phe703Leu;p.Ala990Val</t>
+    <t xml:space="preserve">p.Phe703Leu; p.Ala990Val;  c.1141delA p.Lys383fs</t>
   </si>
   <si>
     <t xml:space="preserve">SP18121</t>
@@ -552,6 +554,7 @@
       <sz val="11"/>
       <name val="Noto Sans CJK SC"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -616,43 +619,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -860,26 +863,24 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="2" width="18.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16381" min="12" style="3" width="8.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16382" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16382" style="4" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="3" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" s="4" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
       <c r="K1" s="1"/>
-      <c r="XFB1" s="0"/>
-      <c r="XFC1" s="0"/>
     </row>
     <row r="2" s="2" customFormat="true" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
@@ -915,8 +916,8 @@
       <c r="K2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="XFB2" s="0"/>
-      <c r="XFC2" s="0"/>
+      <c r="XFB2" s="4"/>
+      <c r="XFC2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
@@ -1513,7 +1514,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="49.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>71</v>
       </c>
@@ -2690,8 +2691,8 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="120"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="120"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2703,90 +2704,90 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>140</v>
       </c>
     </row>

</xml_diff>